<commit_message>
Gespeichert als Strict Open XML-Arbeitsmappe
Änderungen werden anscheinend dennoch nicht in GitHub angezeigt.
</commit_message>
<xml_diff>
--- a/Lärmschadenstool_EXCEL/Lärmschadenstool.xlsx
+++ b/Lärmschadenstool_EXCEL/Lärmschadenstool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
-  <workbookPr codeName="DieseArbeitsmappe"/>
+  <workbookPr dateCompatibility="0" codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dokumente_lokal\GitHub Repository\END2DALY\Lärmschadenstool_EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC11835-95AE-4FCD-86BD-294E2959B9D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{63AA3E00-C5FC-4679-9AD1-7FA2B893E022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,6 +28,9 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -50,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="158">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="299" uniqueCount="158">
   <si>
     <t>L_den</t>
   </si>
@@ -613,7 +616,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.000000"/>
@@ -785,15 +788,15 @@
   </fills>
   <borders count="14">
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4"/>
@@ -801,8 +804,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4" tint="0.499984740745262"/>
@@ -810,8 +813,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.39997558519241921"/>
@@ -819,8 +822,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -828,8 +831,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -837,8 +840,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -848,19 +851,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color indexed="64"/>
-      </left>
-      <right/>
+      </start>
+      <end/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color indexed="64"/>
-      </left>
-      <right/>
+      </start>
+      <end/>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -868,10 +871,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color indexed="64"/>
-      </left>
-      <right/>
+      </start>
+      <end/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -879,10 +882,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color indexed="64"/>
-      </left>
-      <right/>
+      </start>
+      <end/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -892,10 +895,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
+      <start style="thick">
         <color rgb="FFFF0000"/>
-      </left>
-      <right/>
+      </start>
+      <end/>
       <top style="thick">
         <color rgb="FFFF0000"/>
       </top>
@@ -905,8 +908,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top style="thick">
         <color rgb="FFFF0000"/>
       </top>
@@ -916,10 +919,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thick">
+      <start/>
+      <end style="thick">
         <color rgb="FFFF0000"/>
-      </right>
+      </end>
       <top style="thick">
         <color rgb="FFFF0000"/>
       </top>
@@ -1125,6 +1128,27 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1168,27 +1192,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1212,7 +1215,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:a="http://purl.oclc.org/ooxml/drawingml/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -1240,7 +1243,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1284,7 +1287,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1305,7 +1308,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://purl.oclc.org/ooxml/drawingml/spreadsheetDrawing" xmlns:a="http://purl.oclc.org/ooxml/drawingml/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -1333,7 +1336,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1377,7 +1380,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1398,7 +1401,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://purl.oclc.org/ooxml/drawingml/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1517,25 +1520,25 @@
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:lumMod val="110%"/>
+                <a:satMod val="105%"/>
+                <a:tint val="67%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="103%"/>
+                <a:tint val="73%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="109%"/>
+                <a:tint val="81%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1543,25 +1546,25 @@
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:satMod val="103%"/>
+                <a:lumMod val="102%"/>
+                <a:tint val="94%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:satMod val="110%"/>
+                <a:lumMod val="100%"/>
+                <a:shade val="100%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:lumMod val="99%"/>
+                <a:satMod val="120%"/>
+                <a:shade val="78%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1574,21 +1577,21 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1602,7 +1605,7 @@
           <a:effectLst>
             <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="63%"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -1614,32 +1617,32 @@
         </a:solidFill>
         <a:solidFill>
           <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
+            <a:tint val="95%"/>
+            <a:satMod val="170%"/>
           </a:schemeClr>
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="93%"/>
+                <a:satMod val="150%"/>
+                <a:shade val="98%"/>
+                <a:lumMod val="102%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="98%"/>
+                <a:satMod val="130%"/>
+                <a:shade val="90%"/>
+                <a:lumMod val="103%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="63%"/>
+                <a:satMod val="120%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1659,7 +1662,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11457340-40AB-4C39-9488-F3F169CC7A0E}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11457340-40AB-4C39-9488-F3F169CC7A0E}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1668,7 +1671,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D784C34-E246-472E-88D5-CA0D5063A3C9}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D784C34-E246-472E-88D5-CA0D5063A3C9}">
   <sheetPr codeName="Tabelle6"/>
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1678,7 +1681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D71C91-7A22-40CF-B195-068A9D60F08B}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D71C91-7A22-40CF-B195-068A9D60F08B}">
   <sheetPr codeName="Tabelle7"/>
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1688,7 +1691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3AA0BE1-EB71-4657-B503-300F880C587F}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3AA0BE1-EB71-4657-B503-300F880C587F}">
   <dimension ref="A2:A3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1711,7 +1714,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7D27E-13C9-40A4-936B-06BBF9BE4E35}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7D27E-13C9-40A4-936B-06BBF9BE4E35}">
   <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1739,15 +1742,15 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="74.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="120" t="s">
+      <c r="A5" s="133" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="120"/>
-      <c r="C5" s="120"/>
-      <c r="D5" s="120"/>
-      <c r="E5" s="120"/>
-      <c r="F5" s="120"/>
-      <c r="G5" s="120"/>
+      <c r="B5" s="133"/>
+      <c r="C5" s="133"/>
+      <c r="D5" s="133"/>
+      <c r="E5" s="133"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
     </row>
     <row r="8" spans="1:16" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
@@ -1756,10 +1759,10 @@
     </row>
     <row r="9" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="121" t="s">
+      <c r="A10" s="134" t="s">
         <v>155</v>
       </c>
-      <c r="B10" s="121"/>
+      <c r="B10" s="134"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -1769,22 +1772,22 @@
       <c r="B12" s="110" t="s">
         <v>149</v>
       </c>
-      <c r="D12" s="123" t="s">
+      <c r="D12" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="E12" s="123"/>
-      <c r="F12" s="123"/>
-      <c r="G12" s="123"/>
-      <c r="H12" s="123"/>
-      <c r="I12" s="123"/>
-      <c r="K12" s="119" t="s">
+      <c r="E12" s="136"/>
+      <c r="F12" s="136"/>
+      <c r="G12" s="136"/>
+      <c r="H12" s="136"/>
+      <c r="I12" s="136"/>
+      <c r="K12" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="L12" s="119"/>
-      <c r="M12" s="119"/>
-      <c r="N12" s="119"/>
-      <c r="O12" s="119"/>
-      <c r="P12" s="119"/>
+      <c r="L12" s="132"/>
+      <c r="M12" s="132"/>
+      <c r="N12" s="132"/>
+      <c r="O12" s="132"/>
+      <c r="P12" s="132"/>
     </row>
     <row r="13" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="110"/>
@@ -1827,7 +1830,7 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="122" t="s">
+      <c r="A14" s="135" t="s">
         <v>49</v>
       </c>
       <c r="B14" s="110" t="s">
@@ -1874,47 +1877,47 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="122"/>
-      <c r="B15" s="134" t="s">
+      <c r="A15" s="135"/>
+      <c r="B15" s="119" t="s">
         <v>84</v>
       </c>
       <c r="C15" s="15"/>
-      <c r="D15" s="135">
+      <c r="D15" s="120">
         <v>3762100</v>
       </c>
-      <c r="E15" s="135">
+      <c r="E15" s="120">
         <v>3050900</v>
       </c>
-      <c r="F15" s="135">
+      <c r="F15" s="120">
         <v>2479000</v>
       </c>
-      <c r="G15" s="135">
+      <c r="G15" s="120">
         <v>1006400</v>
       </c>
-      <c r="H15" s="135">
+      <c r="H15" s="120">
         <v>99800</v>
       </c>
-      <c r="I15" s="135">
+      <c r="I15" s="120">
         <f t="shared" ref="I15:I23" si="0">SUM(D15:H15)</f>
         <v>10398200</v>
       </c>
-      <c r="J15" s="136"/>
-      <c r="K15" s="137">
+      <c r="J15" s="121"/>
+      <c r="K15" s="122">
         <v>3383500</v>
       </c>
-      <c r="L15" s="137">
+      <c r="L15" s="122">
         <v>2682400</v>
       </c>
-      <c r="M15" s="137">
+      <c r="M15" s="122">
         <v>1283500</v>
       </c>
-      <c r="N15" s="137">
+      <c r="N15" s="122">
         <v>156200</v>
       </c>
-      <c r="O15" s="137">
+      <c r="O15" s="122">
         <v>4900</v>
       </c>
-      <c r="P15" s="137">
+      <c r="P15" s="122">
         <f t="shared" ref="P15:P23" si="1">SUM(K15:O15)</f>
         <v>7510500</v>
       </c>
@@ -1954,7 +1957,7 @@
       <c r="P17" s="109"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="122" t="s">
+      <c r="A18" s="135" t="s">
         <v>78</v>
       </c>
       <c r="B18" s="110" t="s">
@@ -2001,7 +2004,7 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="122"/>
+      <c r="A19" s="135"/>
       <c r="B19" s="110" t="s">
         <v>80</v>
       </c>
@@ -2065,7 +2068,7 @@
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="110"/>
       <c r="B21" s="110"/>
-      <c r="D21" s="138"/>
+      <c r="D21" s="123"/>
       <c r="E21" s="106"/>
       <c r="F21" s="106"/>
       <c r="G21" s="106"/>
@@ -2080,7 +2083,7 @@
       <c r="P21" s="109"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="122" t="s">
+      <c r="A22" s="135" t="s">
         <v>81</v>
       </c>
       <c r="B22" s="110" t="s">
@@ -2127,7 +2130,7 @@
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="122"/>
+      <c r="A23" s="135"/>
       <c r="B23" s="110" t="s">
         <v>83</v>
       </c>
@@ -2178,10 +2181,10 @@
     </row>
     <row r="31" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="121" t="s">
+      <c r="A32" s="134" t="s">
         <v>137</v>
       </c>
-      <c r="B32" s="121"/>
+      <c r="B32" s="134"/>
     </row>
     <row r="33" spans="2:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
@@ -2235,11 +2238,11 @@
       <c r="B39" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C39" s="139">
+      <c r="C39" s="124">
         <f>'Agglomeration road'!C79</f>
         <v>27420.859000423719</v>
       </c>
-      <c r="D39" s="141">
+      <c r="D39" s="126">
         <f>'Agglomeration road'!D79</f>
         <v>308626.30242553435</v>
       </c>
@@ -2248,11 +2251,11 @@
       <c r="B40" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="C40" s="140">
+      <c r="C40" s="125">
         <f>'Agglomeration road'!C80</f>
         <v>1919460130.0296605</v>
       </c>
-      <c r="D40" s="142">
+      <c r="D40" s="127">
         <f>'Agglomeration road'!D80</f>
         <v>21603841169.787403</v>
       </c>
@@ -2274,7 +2277,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FCA578C-B553-47BE-9A2E-931A94425EB8}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FCA578C-B553-47BE-9A2E-931A94425EB8}">
   <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2302,15 +2305,15 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="74.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="120" t="s">
+      <c r="A5" s="133" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="120"/>
-      <c r="C5" s="120"/>
-      <c r="D5" s="120"/>
-      <c r="E5" s="120"/>
-      <c r="F5" s="120"/>
-      <c r="G5" s="120"/>
+      <c r="B5" s="133"/>
+      <c r="C5" s="133"/>
+      <c r="D5" s="133"/>
+      <c r="E5" s="133"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
     </row>
     <row r="8" spans="1:16" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
@@ -2319,10 +2322,10 @@
     </row>
     <row r="9" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="121" t="s">
+      <c r="A10" s="134" t="s">
         <v>155</v>
       </c>
-      <c r="B10" s="121"/>
+      <c r="B10" s="134"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -2332,22 +2335,22 @@
       <c r="B12" s="110" t="s">
         <v>149</v>
       </c>
-      <c r="D12" s="123" t="s">
+      <c r="D12" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="E12" s="123"/>
-      <c r="F12" s="123"/>
-      <c r="G12" s="123"/>
-      <c r="H12" s="123"/>
-      <c r="I12" s="123"/>
-      <c r="K12" s="119" t="s">
+      <c r="E12" s="136"/>
+      <c r="F12" s="136"/>
+      <c r="G12" s="136"/>
+      <c r="H12" s="136"/>
+      <c r="I12" s="136"/>
+      <c r="K12" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="L12" s="119"/>
-      <c r="M12" s="119"/>
-      <c r="N12" s="119"/>
-      <c r="O12" s="119"/>
-      <c r="P12" s="119"/>
+      <c r="L12" s="132"/>
+      <c r="M12" s="132"/>
+      <c r="N12" s="132"/>
+      <c r="O12" s="132"/>
+      <c r="P12" s="132"/>
     </row>
     <row r="13" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="110"/>
@@ -2390,7 +2393,7 @@
       </c>
     </row>
     <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="122" t="s">
+      <c r="A14" s="135" t="s">
         <v>49</v>
       </c>
       <c r="B14" s="110" t="s">
@@ -2437,7 +2440,7 @@
       </c>
     </row>
     <row r="15" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="122"/>
+      <c r="A15" s="135"/>
       <c r="B15" s="111" t="s">
         <v>84</v>
       </c>
@@ -2517,7 +2520,7 @@
       <c r="P17" s="109"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="122" t="s">
+      <c r="A18" s="135" t="s">
         <v>78</v>
       </c>
       <c r="B18" s="110" t="s">
@@ -2564,7 +2567,7 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="122"/>
+      <c r="A19" s="135"/>
       <c r="B19" s="110" t="s">
         <v>80</v>
       </c>
@@ -2628,7 +2631,7 @@
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="110"/>
       <c r="B21" s="110"/>
-      <c r="D21" s="138"/>
+      <c r="D21" s="123"/>
       <c r="E21" s="106"/>
       <c r="F21" s="106"/>
       <c r="G21" s="106"/>
@@ -2643,7 +2646,7 @@
       <c r="P21" s="109"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="122" t="s">
+      <c r="A22" s="135" t="s">
         <v>81</v>
       </c>
       <c r="B22" s="110" t="s">
@@ -2690,7 +2693,7 @@
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="122"/>
+      <c r="A23" s="135"/>
       <c r="B23" s="110" t="s">
         <v>83</v>
       </c>
@@ -2741,10 +2744,10 @@
     </row>
     <row r="31" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="121" t="s">
+      <c r="A32" s="134" t="s">
         <v>137</v>
       </c>
-      <c r="B32" s="121"/>
+      <c r="B32" s="134"/>
     </row>
     <row r="33" spans="2:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
@@ -2798,10 +2801,10 @@
       <c r="B39" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C39" s="143" t="s">
+      <c r="C39" s="128" t="s">
         <v>156</v>
       </c>
-      <c r="D39" s="144" t="s">
+      <c r="D39" s="129" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2809,23 +2812,23 @@
       <c r="B40" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="C40" s="145" t="s">
+      <c r="C40" s="130" t="s">
         <v>156</v>
       </c>
-      <c r="D40" s="146" t="s">
+      <c r="D40" s="131" t="s">
         <v>156</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="K12:P12"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="D12:I12"/>
-    <mergeCell ref="K12:P12"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A18:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2833,7 +2836,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:U88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3345,21 +3348,21 @@
     <row r="39" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C40" s="15"/>
-      <c r="E40" s="124" t="s">
+      <c r="E40" s="137" t="s">
         <v>91</v>
       </c>
-      <c r="F40" s="124"/>
-      <c r="G40" s="124"/>
-      <c r="H40" s="124"/>
-      <c r="I40" s="124"/>
-      <c r="J40" s="124"/>
-      <c r="K40" s="125" t="s">
+      <c r="F40" s="137"/>
+      <c r="G40" s="137"/>
+      <c r="H40" s="137"/>
+      <c r="I40" s="137"/>
+      <c r="J40" s="137"/>
+      <c r="K40" s="138" t="s">
         <v>90</v>
       </c>
-      <c r="L40" s="126"/>
-      <c r="M40" s="126"/>
-      <c r="N40" s="126"/>
-      <c r="O40" s="126"/>
+      <c r="L40" s="139"/>
+      <c r="M40" s="139"/>
+      <c r="N40" s="139"/>
+      <c r="O40" s="139"/>
     </row>
     <row r="41" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="D41" s="15" t="s">
@@ -3400,7 +3403,7 @@
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A42" s="131" t="s">
+      <c r="A42" s="144" t="s">
         <v>101</v>
       </c>
       <c r="B42" s="43" t="s">
@@ -3462,7 +3465,7 @@
       <c r="U42" s="8"/>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A43" s="132"/>
+      <c r="A43" s="145"/>
       <c r="B43" s="15" t="s">
         <v>107</v>
       </c>
@@ -3503,7 +3506,7 @@
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A44" s="133"/>
+      <c r="A44" s="146"/>
       <c r="B44" s="19" t="s">
         <v>108</v>
       </c>
@@ -3577,7 +3580,7 @@
       <c r="O45" s="57"/>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A46" s="131" t="s">
+      <c r="A46" s="144" t="s">
         <v>57</v>
       </c>
       <c r="B46" s="17" t="s">
@@ -3631,7 +3634,7 @@
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A47" s="132"/>
+      <c r="A47" s="145"/>
       <c r="B47" s="15" t="s">
         <v>88</v>
       </c>
@@ -3689,7 +3692,7 @@
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A48" s="132"/>
+      <c r="A48" s="145"/>
       <c r="B48" s="15" t="s">
         <v>110</v>
       </c>
@@ -3714,7 +3717,7 @@
       <c r="O48" s="54"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49" s="133"/>
+      <c r="A49" s="146"/>
       <c r="B49" s="42" t="s">
         <v>145</v>
       </c>
@@ -3739,7 +3742,7 @@
       <c r="O49" s="61"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="131" t="s">
+      <c r="A50" s="144" t="s">
         <v>62</v>
       </c>
       <c r="B50" s="17" t="s">
@@ -3793,7 +3796,7 @@
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51" s="132"/>
+      <c r="A51" s="145"/>
       <c r="B51" s="15" t="s">
         <v>88</v>
       </c>
@@ -3851,7 +3854,7 @@
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" s="132"/>
+      <c r="A52" s="145"/>
       <c r="B52" s="15" t="s">
         <v>110</v>
       </c>
@@ -3876,7 +3879,7 @@
       <c r="O52" s="54"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" s="133"/>
+      <c r="A53" s="146"/>
       <c r="B53" s="42" t="s">
         <v>132</v>
       </c>
@@ -3901,7 +3904,7 @@
       <c r="O53" s="61"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="131" t="s">
+      <c r="A54" s="144" t="s">
         <v>65</v>
       </c>
       <c r="B54" s="17" t="s">
@@ -3955,7 +3958,7 @@
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="132"/>
+      <c r="A55" s="145"/>
       <c r="B55" s="15" t="s">
         <v>88</v>
       </c>
@@ -4013,7 +4016,7 @@
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="132"/>
+      <c r="A56" s="145"/>
       <c r="B56" s="15" t="s">
         <v>110</v>
       </c>
@@ -4038,7 +4041,7 @@
       <c r="O56" s="54"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="133"/>
+      <c r="A57" s="146"/>
       <c r="B57" s="42" t="s">
         <v>133</v>
       </c>
@@ -4063,7 +4066,7 @@
       <c r="O57" s="61"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="131" t="s">
+      <c r="A58" s="144" t="s">
         <v>69</v>
       </c>
       <c r="B58" s="17" t="s">
@@ -4117,7 +4120,7 @@
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="132"/>
+      <c r="A59" s="145"/>
       <c r="B59" s="15" t="s">
         <v>88</v>
       </c>
@@ -4175,7 +4178,7 @@
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="132"/>
+      <c r="A60" s="145"/>
       <c r="B60" s="15" t="s">
         <v>110</v>
       </c>
@@ -4200,7 +4203,7 @@
       <c r="O60" s="54"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A61" s="133"/>
+      <c r="A61" s="146"/>
       <c r="B61" s="42" t="s">
         <v>134</v>
       </c>
@@ -4225,7 +4228,7 @@
       <c r="O61" s="61"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A62" s="129" t="s">
+      <c r="A62" s="142" t="s">
         <v>45</v>
       </c>
       <c r="B62" s="27" t="s">
@@ -4279,7 +4282,7 @@
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A63" s="130"/>
+      <c r="A63" s="143"/>
       <c r="B63" s="27" t="s">
         <v>146</v>
       </c>
@@ -4337,7 +4340,7 @@
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A64" s="128"/>
+      <c r="A64" s="141"/>
       <c r="B64" s="44" t="s">
         <v>147</v>
       </c>
@@ -4383,20 +4386,20 @@
       <c r="B66" s="23"/>
       <c r="C66" s="23"/>
       <c r="D66" s="23"/>
-      <c r="E66" s="124" t="s">
+      <c r="E66" s="137" t="s">
         <v>92</v>
       </c>
-      <c r="F66" s="124"/>
-      <c r="G66" s="124"/>
-      <c r="H66" s="124"/>
-      <c r="I66" s="124"/>
-      <c r="J66" s="125" t="s">
+      <c r="F66" s="137"/>
+      <c r="G66" s="137"/>
+      <c r="H66" s="137"/>
+      <c r="I66" s="137"/>
+      <c r="J66" s="138" t="s">
         <v>93</v>
       </c>
-      <c r="K66" s="126"/>
-      <c r="L66" s="126"/>
-      <c r="M66" s="126"/>
-      <c r="N66" s="126"/>
+      <c r="K66" s="139"/>
+      <c r="L66" s="139"/>
+      <c r="M66" s="139"/>
+      <c r="N66" s="139"/>
       <c r="O66" s="24"/>
     </row>
     <row r="67" spans="1:15" ht="30" x14ac:dyDescent="0.25">
@@ -4439,7 +4442,7 @@
       <c r="O67" s="15"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A68" s="131" t="s">
+      <c r="A68" s="144" t="s">
         <v>101</v>
       </c>
       <c r="B68" s="18" t="s">
@@ -4493,7 +4496,7 @@
       <c r="O68" s="15"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="132"/>
+      <c r="A69" s="145"/>
       <c r="B69" s="15" t="s">
         <v>107</v>
       </c>
@@ -4532,7 +4535,7 @@
       <c r="O69" s="15"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A70" s="133"/>
+      <c r="A70" s="146"/>
       <c r="B70" s="19" t="s">
         <v>108</v>
       </c>
@@ -4604,7 +4607,7 @@
       <c r="O71" s="15"/>
     </row>
     <row r="72" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="127" t="s">
+      <c r="A72" s="140" t="s">
         <v>53</v>
       </c>
       <c r="B72" s="27" t="s">
@@ -4654,7 +4657,7 @@
       </c>
     </row>
     <row r="73" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="127"/>
+      <c r="A73" s="140"/>
       <c r="B73" s="27" t="s">
         <v>146</v>
       </c>
@@ -4708,7 +4711,7 @@
       </c>
     </row>
     <row r="74" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="128"/>
+      <c r="A74" s="141"/>
       <c r="B74" s="44" t="s">
         <v>148</v>
       </c>
@@ -4858,7 +4861,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1B57BF-B5FC-49D0-8C1C-84AA1C3FC65A}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1B57BF-B5FC-49D0-8C1C-84AA1C3FC65A}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4938,7 +4941,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A8C717-7812-4473-9D8B-3495A5B0BB7F}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A8C717-7812-4473-9D8B-3495A5B0BB7F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -4948,7 +4951,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3BA502-77FB-4AA9-A654-F467290EB112}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3BA502-77FB-4AA9-A654-F467290EB112}">
   <sheetPr codeName="Tabelle2"/>
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5137,7 +5140,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{601D2B11-F41E-4CFB-A90C-BC8CA1A15B8D}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{601D2B11-F41E-4CFB-A90C-BC8CA1A15B8D}">
   <sheetPr codeName="Tabelle3"/>
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5147,7 +5150,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D15C0212-0B91-4E6B-BA83-4D03E3220F57}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D15C0212-0B91-4E6B-BA83-4D03E3220F57}">
   <sheetPr codeName="Tabelle5"/>
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>